<commit_message>
Equity sheet: founder name cells are live refs to Inputs
</commit_message>
<xml_diff>
--- a/examples/meetingroi.xlsx
+++ b/examples/meetingroi.xlsx
@@ -4541,10 +4541,9 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Founder A</t>
-        </is>
+      <c r="A5">
+        <f>Inputs!$B$80</f>
+        <v/>
       </c>
       <c r="B5" s="18">
         <f>in_founder1_time_pct</f>
@@ -4576,10 +4575,9 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Founder B</t>
-        </is>
+      <c r="A6">
+        <f>Inputs!$B$86</f>
+        <v/>
       </c>
       <c r="B6" s="18">
         <f>in_founder2_time_pct</f>
@@ -4611,10 +4609,9 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Founder C</t>
-        </is>
+      <c r="A7">
+        <f>Inputs!$B$92</f>
+        <v/>
       </c>
       <c r="B7" s="18">
         <f>in_founder3_time_pct</f>
@@ -4646,10 +4643,9 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Founder D</t>
-        </is>
+      <c r="A8">
+        <f>Inputs!$B$98</f>
+        <v/>
       </c>
       <c r="B8" s="18">
         <f>in_founder4_time_pct</f>

</xml_diff>

<commit_message>
Embed cached values for every formula cell
openpyxl never evaluates formulas, so xlsx files it writes have empty <v>
elements. Apps that don't honor fullCalcOnLoad (Apple Numbers, Google Sheets
import) show all formula cells as blank — and even after editing inputs, they
don't recompute.

After saving, use the 'formulas' package to evaluate every cell and inject
the result alongside the existing <f> formula. Cells now serialize as
<c><f>FORMULA</f><v>VALUE</v></c>, so:
  - On open in any app: values display immediately
  - On edit in Excel: formulas recompute live (was already working)
  - On edit in Numbers: at minimum, initial values are correct (Numbers will
    recompute edited cells; some chains may need explicit recalc)

Also fixes regex bug in rels parsing where Target paths containing '/' broke
the sheet-name-to-XML-file map, so the injection silently did nothing.
</commit_message>
<xml_diff>
--- a/examples/meetingroi.xlsx
+++ b/examples/meetingroi.xlsx
@@ -626,7 +626,7 @@
       </c>
       <c r="B4" s="3">
         <f>Scorecard!C16</f>
-        <v/>
+        <v>3.640463498</v>
       </c>
     </row>
     <row r="5">
@@ -637,7 +637,7 @@
       </c>
       <c r="B5" s="4">
         <f>Scorecard!C17</f>
-        <v/>
+        <v>66.01158745</v>
       </c>
     </row>
     <row r="6">
@@ -646,9 +646,9 @@
           <t>Verdict</t>
         </is>
       </c>
-      <c r="B6">
+      <c r="B6" t="str">
         <f>Scorecard!C18</f>
-        <v/>
+        <v>GO</v>
       </c>
     </row>
     <row r="8">
@@ -659,7 +659,7 @@
       </c>
       <c r="B8" s="5">
         <f>Valuation_DCF!B19</f>
-        <v/>
+        <v>2445239.896</v>
       </c>
     </row>
     <row r="9">
@@ -670,7 +670,7 @@
       </c>
       <c r="B9" s="5">
         <f>Valuation_Comps!B5</f>
-        <v/>
+        <v>6120000</v>
       </c>
     </row>
     <row r="10">
@@ -681,7 +681,7 @@
       </c>
       <c r="B10" s="5">
         <f>Valuation_EarlyStage!B3</f>
-        <v/>
+        <v>1550000</v>
       </c>
     </row>
     <row r="11">
@@ -692,7 +692,7 @@
       </c>
       <c r="B11" s="5">
         <f>Valuation_EarlyStage!B4</f>
-        <v/>
+        <v>6067439.163</v>
       </c>
     </row>
     <row r="12">
@@ -703,7 +703,7 @@
       </c>
       <c r="B12" s="5">
         <f>Valuation_EarlyStage!B5</f>
-        <v/>
+        <v>16666666.67</v>
       </c>
     </row>
     <row r="13">
@@ -714,7 +714,7 @@
       </c>
       <c r="B13" s="5">
         <f>Valuation_EarlyStage!B9</f>
-        <v/>
+        <v>4823809.974</v>
       </c>
     </row>
     <row r="14">
@@ -725,7 +725,7 @@
       </c>
       <c r="B14" s="5">
         <f>Valuation_Patent!B7</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -736,7 +736,7 @@
       </c>
       <c r="B16" s="5">
         <f>Org!I23</f>
-        <v/>
+        <v>948000</v>
       </c>
     </row>
     <row r="17">
@@ -747,7 +747,7 @@
       </c>
       <c r="B17" s="5">
         <f>Org!J23</f>
-        <v/>
+        <v>4236000</v>
       </c>
     </row>
   </sheetData>
@@ -871,7 +871,7 @@
       </c>
       <c r="B14" s="24">
         <f>(B4*B5*B6*B7*B8*B9)/(B10*B11)</f>
-        <v/>
+        <v>30</v>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
@@ -887,7 +887,7 @@
       </c>
       <c r="B15" s="4">
         <f>(MIN(100,B4*B5*B8/100000)+MAX(0,MIN(1,1/MAX(B9,0.5)))*100+B6*100)/B10</f>
-        <v/>
+        <v>106.6666667</v>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
       </c>
       <c r="B16" s="5">
         <f>(B4*B5*B8)/B10</f>
-        <v/>
+        <v>12000000</v>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
@@ -919,7 +919,7 @@
       </c>
       <c r="B17" s="5">
         <f>B8*(B4*B5)*B9-B11</f>
-        <v/>
+        <v>71040000</v>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
@@ -2602,7 +2602,7 @@
       </c>
       <c r="C4" s="3">
         <f>AVERAGE(in_score_problem_severity,in_score_problem_frequency,in_score_willingness_to_pay)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="C5" s="3">
         <f>AVERAGE(in_score_market_timing)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="C6" s="3">
         <f>AVERAGE(in_score_moat_tech,in_score_moat_data,in_score_moat_brand,in_score_ip_strength)</f>
-        <v/>
+        <v>2.25</v>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
@@ -2659,7 +2659,7 @@
       </c>
       <c r="C7" s="3">
         <f>AVERAGE(in_score_team_domain,in_score_team_execution,in_score_team_completeness)</f>
-        <v/>
+        <v>3.333333333</v>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
       </c>
       <c r="C8" s="3">
         <f>AVERAGE(in_score_gtm_clarity)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="C9" s="3">
         <f>AVERAGE(in_score_unit_economics,in_score_capital_efficiency)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="C10" s="3">
         <f>AVERAGE(in_score_scalability)</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="C11" s="3">
         <f>AVERAGE(in_score_regulatory_risk)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="C12" s="3">
         <f>AVERAGE(in_score_ai_resilience)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
@@ -2770,7 +2770,7 @@
       </c>
       <c r="C14" s="3">
         <f>SUMPRODUCT(B4:B12,C4:C12)</f>
-        <v/>
+        <v>3.505</v>
       </c>
     </row>
     <row r="15">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="C15" s="3">
         <f>MAX(-1,MIN(1,LOG10(MAX(1,in_tam_usd)/1000000000)))*0.15</f>
-        <v/>
+        <v>0.135463498</v>
       </c>
     </row>
     <row r="16">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="C16" s="3">
         <f>MAX(1,MIN(5,C14+C15))</f>
-        <v/>
+        <v>3.640463498</v>
       </c>
     </row>
     <row r="17">
@@ -2803,7 +2803,7 @@
       </c>
       <c r="C17" s="4">
         <f>(C16-1)/4*100</f>
-        <v/>
+        <v>66.01158745</v>
       </c>
     </row>
     <row r="18">
@@ -2812,9 +2812,9 @@
           <t>Verdict</t>
         </is>
       </c>
-      <c r="C18">
+      <c r="C18" t="str">
         <f>IF(C17&gt;=75,"STRONG GO",IF(C17&gt;=60,"GO",IF(C17&gt;=45,"CONDITIONAL",IF(C17&gt;=30,"WEAK","NO-GO"))))</f>
-        <v/>
+        <v>GO</v>
       </c>
     </row>
   </sheetData>
@@ -2920,15 +2920,15 @@
       </c>
       <c r="D4">
         <f>ROUND(1.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="E4">
         <f>ROUND(1.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>1.2</v>
       </c>
       <c r="F4" s="18">
         <f>ROUND(0.2*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.34</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2942,11 +2942,11 @@
       </c>
       <c r="I4" s="5">
         <f>D4*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>72000</v>
       </c>
       <c r="J4" s="5">
         <f>E4*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>144000</v>
       </c>
     </row>
     <row r="5">
@@ -2967,15 +2967,15 @@
       </c>
       <c r="D5">
         <f>ROUND(1.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="E5">
         <f>ROUND(1.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>1.2</v>
       </c>
       <c r="F5" s="18">
         <f>ROUND(0.3*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.41</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -2989,11 +2989,11 @@
       </c>
       <c r="I5" s="5">
         <f>D5*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>72000</v>
       </c>
       <c r="J5" s="5">
         <f>E5*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>144000</v>
       </c>
     </row>
     <row r="6">
@@ -3014,15 +3014,15 @@
       </c>
       <c r="D6">
         <f>ROUND(0.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E6">
         <f>ROUND(1.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>1.2</v>
       </c>
       <c r="F6" s="18">
         <f>ROUND(0.4*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.48</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -3036,11 +3036,11 @@
       </c>
       <c r="I6" s="5">
         <f>D6*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J6" s="5">
         <f>E6*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>144000</v>
       </c>
     </row>
     <row r="7">
@@ -3061,15 +3061,15 @@
       </c>
       <c r="D7">
         <f>ROUND(0.5/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.3</v>
       </c>
       <c r="E7">
         <f>ROUND(1.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>1.2</v>
       </c>
       <c r="F7" s="18">
         <f>ROUND(0.3*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.41</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -3083,11 +3083,11 @@
       </c>
       <c r="I7" s="5">
         <f>D7*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>36000</v>
       </c>
       <c r="J7" s="5">
         <f>E7*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>144000</v>
       </c>
     </row>
     <row r="8">
@@ -3108,15 +3108,15 @@
       </c>
       <c r="D8">
         <f>ROUND(1.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="E8">
         <f>ROUND(2.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>2.3</v>
       </c>
       <c r="F8" s="18">
         <f>ROUND(0.4*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.48</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -3130,11 +3130,11 @@
       </c>
       <c r="I8" s="5">
         <f>D8*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>72000</v>
       </c>
       <c r="J8" s="5">
         <f>E8*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>276000</v>
       </c>
     </row>
     <row r="9">
@@ -3155,15 +3155,15 @@
       </c>
       <c r="D9">
         <f>ROUND(1.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="E9">
         <f>ROUND(2.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>2.3</v>
       </c>
       <c r="F9" s="18">
         <f>ROUND(0.5*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.54</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -3177,11 +3177,11 @@
       </c>
       <c r="I9" s="5">
         <f>D9*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>72000</v>
       </c>
       <c r="J9" s="5">
         <f>E9*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>276000</v>
       </c>
     </row>
     <row r="10">
@@ -3202,15 +3202,15 @@
       </c>
       <c r="D10">
         <f>ROUND(1.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="E10">
         <f>ROUND(1.5/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>1.8</v>
       </c>
       <c r="F10" s="18">
         <f>ROUND(0.25*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.37</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -3224,11 +3224,11 @@
       </c>
       <c r="I10" s="5">
         <f>D10*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>72000</v>
       </c>
       <c r="J10" s="5">
         <f>E10*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>216000</v>
       </c>
     </row>
     <row r="11">
@@ -3249,15 +3249,15 @@
       </c>
       <c r="D11">
         <f>ROUND(2.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>1.2</v>
       </c>
       <c r="E11">
         <f>ROUND(4.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>4.7</v>
       </c>
       <c r="F11" s="18">
         <f>ROUND(0.55*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.58</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -3271,11 +3271,11 @@
       </c>
       <c r="I11" s="5">
         <f>D11*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>144000</v>
       </c>
       <c r="J11" s="5">
         <f>E11*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>564000</v>
       </c>
     </row>
     <row r="12">
@@ -3296,15 +3296,15 @@
       </c>
       <c r="D12">
         <f>ROUND(1.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="E12">
         <f>ROUND(2.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>2.3</v>
       </c>
       <c r="F12" s="18">
         <f>ROUND(0.4*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.48</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -3318,11 +3318,11 @@
       </c>
       <c r="I12" s="5">
         <f>D12*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>72000</v>
       </c>
       <c r="J12" s="5">
         <f>E12*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>276000</v>
       </c>
     </row>
     <row r="13">
@@ -3343,15 +3343,15 @@
       </c>
       <c r="D13">
         <f>ROUND(0.5/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.3</v>
       </c>
       <c r="E13">
         <f>ROUND(1.5/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>1.8</v>
       </c>
       <c r="F13" s="18">
         <f>ROUND(0.6*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.62</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -3365,11 +3365,11 @@
       </c>
       <c r="I13" s="5">
         <f>D13*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>36000</v>
       </c>
       <c r="J13" s="5">
         <f>E13*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>216000</v>
       </c>
     </row>
     <row r="14">
@@ -3390,15 +3390,15 @@
       </c>
       <c r="D14">
         <f>ROUND(0.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E14">
         <f>ROUND(1.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>1.2</v>
       </c>
       <c r="F14" s="18">
         <f>ROUND(0.7*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.69</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -3412,11 +3412,11 @@
       </c>
       <c r="I14" s="5">
         <f>D14*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J14" s="5">
         <f>E14*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>144000</v>
       </c>
     </row>
     <row r="15">
@@ -3437,15 +3437,15 @@
       </c>
       <c r="D15">
         <f>ROUND(0.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E15">
         <f>ROUND(1.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>1.2</v>
       </c>
       <c r="F15" s="18">
         <f>ROUND(0.5*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.54</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -3459,11 +3459,11 @@
       </c>
       <c r="I15" s="5">
         <f>D15*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J15" s="5">
         <f>E15*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>144000</v>
       </c>
     </row>
     <row r="16">
@@ -3484,15 +3484,15 @@
       </c>
       <c r="D16">
         <f>ROUND(0.5/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.3</v>
       </c>
       <c r="E16">
         <f>ROUND(1.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>1.2</v>
       </c>
       <c r="F16" s="18">
         <f>ROUND(0.3*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.41</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3506,11 +3506,11 @@
       </c>
       <c r="I16" s="5">
         <f>D16*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>36000</v>
       </c>
       <c r="J16" s="5">
         <f>E16*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>144000</v>
       </c>
     </row>
     <row r="17">
@@ -3531,15 +3531,15 @@
       </c>
       <c r="D17">
         <f>ROUND(1.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="E17">
         <f>ROUND(3.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>3.5</v>
       </c>
       <c r="F17" s="18">
         <f>ROUND(0.4*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.48</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -3553,11 +3553,11 @@
       </c>
       <c r="I17" s="5">
         <f>D17*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>72000</v>
       </c>
       <c r="J17" s="5">
         <f>E17*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>420000</v>
       </c>
     </row>
     <row r="18">
@@ -3578,15 +3578,15 @@
       </c>
       <c r="D18">
         <f>ROUND(1.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="E18">
         <f>ROUND(2.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>2.3</v>
       </c>
       <c r="F18" s="18">
         <f>ROUND(0.6*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.62</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -3600,11 +3600,11 @@
       </c>
       <c r="I18" s="5">
         <f>D18*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>72000</v>
       </c>
       <c r="J18" s="5">
         <f>E18*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>276000</v>
       </c>
     </row>
     <row r="19">
@@ -3625,15 +3625,15 @@
       </c>
       <c r="D19">
         <f>ROUND(1.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="E19">
         <f>ROUND(2.5/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>2.9</v>
       </c>
       <c r="F19" s="18">
         <f>ROUND(0.55*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.58</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -3647,11 +3647,11 @@
       </c>
       <c r="I19" s="5">
         <f>D19*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>72000</v>
       </c>
       <c r="J19" s="5">
         <f>E19*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>348000</v>
       </c>
     </row>
     <row r="20">
@@ -3672,15 +3672,15 @@
       </c>
       <c r="D20">
         <f>ROUND(0.0/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E20">
         <f>ROUND(1.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>1.2</v>
       </c>
       <c r="F20" s="18">
         <f>ROUND(0.65*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.65</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -3694,11 +3694,11 @@
       </c>
       <c r="I20" s="5">
         <f>D20*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J20" s="5">
         <f>E20*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>144000</v>
       </c>
     </row>
     <row r="21">
@@ -3719,15 +3719,15 @@
       </c>
       <c r="D21">
         <f>ROUND(0.5/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.3</v>
       </c>
       <c r="E21">
         <f>ROUND(1.0/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>1.2</v>
       </c>
       <c r="F21" s="18">
         <f>ROUND(0.5*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.54</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -3741,11 +3741,11 @@
       </c>
       <c r="I21" s="5">
         <f>D21*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>36000</v>
       </c>
       <c r="J21" s="5">
         <f>E21*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>144000</v>
       </c>
     </row>
     <row r="22">
@@ -3766,15 +3766,15 @@
       </c>
       <c r="D22">
         <f>ROUND(0.2/13.2*in_target_headcount_y1,1)</f>
-        <v/>
+        <v>0.1</v>
       </c>
       <c r="E22">
         <f>ROUND(0.5/30.0*in_target_headcount_y3,1)</f>
-        <v/>
+        <v>0.6</v>
       </c>
       <c r="F22" s="18">
         <f>ROUND(0.55*0.7+in_ai_automation_target*0.3,2)</f>
-        <v/>
+        <v>0.58</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -3788,11 +3788,11 @@
       </c>
       <c r="I22" s="5">
         <f>D22*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>12000</v>
       </c>
       <c r="J22" s="5">
         <f>E22*in_avg_fully_loaded_cost</f>
-        <v/>
+        <v>72000</v>
       </c>
     </row>
     <row r="23">
@@ -3803,19 +3803,19 @@
       </c>
       <c r="D23" s="4">
         <f>SUM(D4:D22)</f>
-        <v/>
+        <v>7.9</v>
       </c>
       <c r="E23" s="4">
         <f>SUM(E4:E22)</f>
-        <v/>
+        <v>35.3</v>
       </c>
       <c r="I23" s="5">
         <f>SUM(I4:I22)</f>
-        <v/>
+        <v>948000</v>
       </c>
       <c r="J23" s="5">
         <f>SUM(J4:J22)</f>
-        <v/>
+        <v>4236000</v>
       </c>
     </row>
   </sheetData>
@@ -3887,23 +3887,23 @@
       </c>
       <c r="B4" s="5">
         <f>in_rev_y1</f>
-        <v/>
+        <v>240000</v>
       </c>
       <c r="C4" s="5">
         <f>B4*(1+in_rev_growth_y2)</f>
-        <v/>
+        <v>960000</v>
       </c>
       <c r="D4" s="5">
         <f>C4*(1+in_rev_growth_y3)</f>
-        <v/>
+        <v>2880000</v>
       </c>
       <c r="E4" s="5">
         <f>D4*(1+in_rev_growth_y4)</f>
-        <v/>
+        <v>6336000</v>
       </c>
       <c r="F4" s="5">
         <f>E4*(1+in_rev_growth_y5)</f>
-        <v/>
+        <v>10771200</v>
       </c>
     </row>
     <row r="5">
@@ -3914,23 +3914,23 @@
       </c>
       <c r="B5" s="5">
         <f>B4*in_gross_margin</f>
-        <v/>
+        <v>187200</v>
       </c>
       <c r="C5" s="5">
         <f>C4*in_gross_margin</f>
-        <v/>
+        <v>748800</v>
       </c>
       <c r="D5" s="5">
         <f>D4*in_gross_margin</f>
-        <v/>
+        <v>2246400</v>
       </c>
       <c r="E5" s="5">
         <f>E4*in_gross_margin</f>
-        <v/>
+        <v>4942080</v>
       </c>
       <c r="F5" s="5">
         <f>F4*in_gross_margin</f>
-        <v/>
+        <v>8401536</v>
       </c>
     </row>
     <row r="6">
@@ -3941,23 +3941,23 @@
       </c>
       <c r="B6" s="5">
         <f>B4*in_opex_pct_rev</f>
-        <v/>
+        <v>132000</v>
       </c>
       <c r="C6" s="5">
         <f>C4*in_opex_pct_rev</f>
-        <v/>
+        <v>528000</v>
       </c>
       <c r="D6" s="5">
         <f>D4*in_opex_pct_rev</f>
-        <v/>
+        <v>1584000</v>
       </c>
       <c r="E6" s="5">
         <f>E4*in_opex_pct_rev</f>
-        <v/>
+        <v>3484800</v>
       </c>
       <c r="F6" s="5">
         <f>F4*in_opex_pct_rev</f>
-        <v/>
+        <v>5924160</v>
       </c>
     </row>
     <row r="7">
@@ -3968,23 +3968,23 @@
       </c>
       <c r="B7" s="5">
         <f>B5-B6</f>
-        <v/>
+        <v>55200</v>
       </c>
       <c r="C7" s="5">
         <f>C5-C6</f>
-        <v/>
+        <v>220800</v>
       </c>
       <c r="D7" s="5">
         <f>D5-D6</f>
-        <v/>
+        <v>662400</v>
       </c>
       <c r="E7" s="5">
         <f>E5-E6</f>
-        <v/>
+        <v>1457280</v>
       </c>
       <c r="F7" s="5">
         <f>F5-F6</f>
-        <v/>
+        <v>2477376</v>
       </c>
     </row>
     <row r="8">
@@ -3995,23 +3995,23 @@
       </c>
       <c r="B8" s="5">
         <f>B7*(1-in_tax_rate)</f>
-        <v/>
+        <v>41400</v>
       </c>
       <c r="C8" s="5">
         <f>C7*(1-in_tax_rate)</f>
-        <v/>
+        <v>165600</v>
       </c>
       <c r="D8" s="5">
         <f>D7*(1-in_tax_rate)</f>
-        <v/>
+        <v>496800</v>
       </c>
       <c r="E8" s="5">
         <f>E7*(1-in_tax_rate)</f>
-        <v/>
+        <v>1092960</v>
       </c>
       <c r="F8" s="5">
         <f>F7*(1-in_tax_rate)</f>
-        <v/>
+        <v>1858032</v>
       </c>
     </row>
     <row r="9">
@@ -4022,23 +4022,23 @@
       </c>
       <c r="B9" s="5">
         <f>B4*in_capex_pct_rev</f>
-        <v/>
+        <v>4800</v>
       </c>
       <c r="C9" s="5">
         <f>C4*in_capex_pct_rev</f>
-        <v/>
+        <v>19200</v>
       </c>
       <c r="D9" s="5">
         <f>D4*in_capex_pct_rev</f>
-        <v/>
+        <v>57600</v>
       </c>
       <c r="E9" s="5">
         <f>E4*in_capex_pct_rev</f>
-        <v/>
+        <v>126720</v>
       </c>
       <c r="F9" s="5">
         <f>F4*in_capex_pct_rev</f>
-        <v/>
+        <v>215424</v>
       </c>
     </row>
     <row r="10">
@@ -4049,23 +4049,23 @@
       </c>
       <c r="B10" s="5">
         <f>B4*in_nwc_pct_rev</f>
-        <v/>
+        <v>9600</v>
       </c>
       <c r="C10" s="5">
         <f>C4*in_nwc_pct_rev</f>
-        <v/>
+        <v>38400</v>
       </c>
       <c r="D10" s="5">
         <f>D4*in_nwc_pct_rev</f>
-        <v/>
+        <v>115200</v>
       </c>
       <c r="E10" s="5">
         <f>E4*in_nwc_pct_rev</f>
-        <v/>
+        <v>253440</v>
       </c>
       <c r="F10" s="5">
         <f>F4*in_nwc_pct_rev</f>
-        <v/>
+        <v>430848</v>
       </c>
     </row>
     <row r="11">
@@ -4076,23 +4076,23 @@
       </c>
       <c r="B11" s="5">
         <f>B10</f>
-        <v/>
+        <v>9600</v>
       </c>
       <c r="C11" s="5">
         <f>C10-B10</f>
-        <v/>
+        <v>28800</v>
       </c>
       <c r="D11" s="5">
         <f>D10-C10</f>
-        <v/>
+        <v>76800</v>
       </c>
       <c r="E11" s="5">
         <f>E10-D10</f>
-        <v/>
+        <v>138240</v>
       </c>
       <c r="F11" s="5">
         <f>F10-E10</f>
-        <v/>
+        <v>177408</v>
       </c>
     </row>
     <row r="12">
@@ -4103,23 +4103,23 @@
       </c>
       <c r="B12" s="5">
         <f>B8-B9-B11</f>
-        <v/>
+        <v>27000</v>
       </c>
       <c r="C12" s="5">
         <f>C8-C9-C11</f>
-        <v/>
+        <v>117600</v>
       </c>
       <c r="D12" s="5">
         <f>D8-D9-D11</f>
-        <v/>
+        <v>362400</v>
       </c>
       <c r="E12" s="5">
         <f>E8-E9-E11</f>
-        <v/>
+        <v>828000</v>
       </c>
       <c r="F12" s="5">
         <f>F8-F9-F11</f>
-        <v/>
+        <v>1465200</v>
       </c>
     </row>
     <row r="13">
@@ -4130,23 +4130,23 @@
       </c>
       <c r="B13" s="19">
         <f>1/(1+in_discount_rate)^1</f>
-        <v/>
+        <v>0.7692307692</v>
       </c>
       <c r="C13" s="19">
         <f>1/(1+in_discount_rate)^2</f>
-        <v/>
+        <v>0.5917159763</v>
       </c>
       <c r="D13" s="19">
         <f>1/(1+in_discount_rate)^3</f>
-        <v/>
+        <v>0.4551661356</v>
       </c>
       <c r="E13" s="19">
         <f>1/(1+in_discount_rate)^4</f>
-        <v/>
+        <v>0.3501277966</v>
       </c>
       <c r="F13" s="19">
         <f>1/(1+in_discount_rate)^5</f>
-        <v/>
+        <v>0.2693290743</v>
       </c>
     </row>
     <row r="14">
@@ -4157,23 +4157,23 @@
       </c>
       <c r="B14" s="5">
         <f>B12*B13</f>
-        <v/>
+        <v>20769.23077</v>
       </c>
       <c r="C14" s="5">
         <f>C12*C13</f>
-        <v/>
+        <v>69585.79882</v>
       </c>
       <c r="D14" s="5">
         <f>D12*D13</f>
-        <v/>
+        <v>164952.2076</v>
       </c>
       <c r="E14" s="5">
         <f>E12*E13</f>
-        <v/>
+        <v>289905.8156</v>
       </c>
       <c r="F14" s="5">
         <f>F12*F13</f>
-        <v/>
+        <v>394620.9597</v>
       </c>
     </row>
     <row r="16">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="B16" s="5">
         <f>F12*(1+in_terminal_growth)/(in_discount_rate-in_terminal_growth)</f>
-        <v/>
+        <v>5589466.667</v>
       </c>
     </row>
     <row r="17">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="B17" s="5">
         <f>B16/(1+in_discount_rate)^5</f>
-        <v/>
+        <v>1505405.883</v>
       </c>
     </row>
     <row r="18">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="B18" s="5">
         <f>SUM(B14:F14)+B17</f>
-        <v/>
+        <v>2445239.896</v>
       </c>
     </row>
     <row r="19">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="B19" s="5">
         <f>B18-in_net_debt_usd</f>
-        <v/>
+        <v>2445239.896</v>
       </c>
     </row>
   </sheetData>
@@ -4253,7 +4253,7 @@
       </c>
       <c r="B3" s="5">
         <f>in_comp_rev_multiple*in_comp_ntm_revenue</f>
-        <v/>
+        <v>9600000</v>
       </c>
     </row>
     <row r="4">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="B4" s="5">
         <f>in_comp_ebitda_multiple*in_comp_ntm_ebitda</f>
-        <v/>
+        <v>2640000</v>
       </c>
     </row>
     <row r="5">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="B5" s="5">
         <f>AVERAGE(B3:B4)</f>
-        <v/>
+        <v>6120000</v>
       </c>
     </row>
   </sheetData>
@@ -4311,7 +4311,7 @@
       </c>
       <c r="B3" s="5">
         <f>in_berkus_idea+in_berkus_prototype+in_berkus_team+in_berkus_relationships+in_berkus_sales</f>
-        <v/>
+        <v>1550000</v>
       </c>
     </row>
     <row r="4">
@@ -4322,7 +4322,7 @@
       </c>
       <c r="B4" s="5">
         <f>in_scorecard_avg_premoney*Scorecard!C16/3</f>
-        <v/>
+        <v>6067439.163</v>
       </c>
     </row>
     <row r="5">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="B5" s="5">
         <f>in_vc_exit_value/in_vc_target_roi</f>
-        <v/>
+        <v>16666666.67</v>
       </c>
     </row>
     <row r="6">
@@ -4344,7 +4344,7 @@
       </c>
       <c r="B6" s="5">
         <f>MAX(Valuation_DCF!B19,Valuation_Comps!B5)*1.5</f>
-        <v/>
+        <v>9180000</v>
       </c>
     </row>
     <row r="7">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="B7" s="5">
         <f>AVERAGE(Valuation_DCF!B19,Valuation_Comps!B5)</f>
-        <v/>
+        <v>4282619.948</v>
       </c>
     </row>
     <row r="8">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="B8" s="5">
         <f>B3</f>
-        <v/>
+        <v>1550000</v>
       </c>
     </row>
     <row r="9">
@@ -4377,7 +4377,7 @@
       </c>
       <c r="B9" s="5">
         <f>0.25*B6+0.5*B7+0.25*B8</f>
-        <v/>
+        <v>4823809.974</v>
       </c>
     </row>
   </sheetData>
@@ -4413,7 +4413,7 @@
       </c>
       <c r="B3" s="5">
         <f>in_patent_dev_cost_usd</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="B4" s="5">
         <f>in_patent_comparable_sale_usd</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="B5" s="5">
         <f>in_patent_royalty_rate*in_patent_revenue_attributable*(1-(1+in_discount_rate)^-in_patent_useful_life_years)/in_discount_rate</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="B6" s="5">
         <f>0.20*in_patent_revenue_attributable*(1-(1+in_discount_rate)^-in_patent_useful_life_years)/in_discount_rate</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="B7" s="5">
         <f>AVERAGE(B3:B6)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4541,139 +4541,139 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5">
+      <c r="A5" t="str">
         <f>Inputs!$B$80</f>
-        <v/>
+        <v>Founder A</v>
       </c>
       <c r="B5" s="18">
         <f>in_founder1_time_pct</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="C5" s="5">
         <f>in_founder1_salary_forgone_usd</f>
-        <v/>
+        <v>100000</v>
       </c>
       <c r="D5" s="5">
         <f>in_founder1_capital_usd</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E5">
         <f>in_founder1_ip_score</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F5">
         <f>in_founder1_role_criticality</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G5" s="5">
         <f>B5*C5+D5+E5*100000+F5*50000</f>
-        <v/>
+        <v>600000</v>
       </c>
       <c r="H5" s="20">
         <f>IF($G$9=0,0,G5/$G$9*(1-in_esop_pool_pct))</f>
-        <v/>
+        <v>0.425</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6">
+      <c r="A6" t="str">
         <f>Inputs!$B$86</f>
-        <v/>
+        <v>Founder B</v>
       </c>
       <c r="B6" s="18">
         <f>in_founder2_time_pct</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="C6" s="5">
         <f>in_founder2_salary_forgone_usd</f>
-        <v/>
+        <v>100000</v>
       </c>
       <c r="D6" s="5">
         <f>in_founder2_capital_usd</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E6">
         <f>in_founder2_ip_score</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F6">
         <f>in_founder2_role_criticality</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G6" s="5">
         <f>B6*C6+D6+E6*100000+F6*50000</f>
-        <v/>
+        <v>600000</v>
       </c>
       <c r="H6" s="20">
         <f>IF($G$9=0,0,G6/$G$9*(1-in_esop_pool_pct))</f>
-        <v/>
+        <v>0.425</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7">
+      <c r="A7" t="str">
         <f>Inputs!$B$92</f>
-        <v/>
+        <v>Founder C</v>
       </c>
       <c r="B7" s="18">
         <f>in_founder3_time_pct</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C7" s="5">
         <f>in_founder3_salary_forgone_usd</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D7" s="5">
         <f>in_founder3_capital_usd</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E7">
         <f>in_founder3_ip_score</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F7">
         <f>in_founder3_role_criticality</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G7" s="5">
         <f>B7*C7+D7+E7*100000+F7*50000</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H7" s="20">
         <f>IF($G$9=0,0,G7/$G$9*(1-in_esop_pool_pct))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8">
+      <c r="A8" t="str">
         <f>Inputs!$B$98</f>
-        <v/>
+        <v>Founder D</v>
       </c>
       <c r="B8" s="18">
         <f>in_founder4_time_pct</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C8" s="5">
         <f>in_founder4_salary_forgone_usd</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D8" s="5">
         <f>in_founder4_capital_usd</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E8">
         <f>in_founder4_ip_score</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F8">
         <f>in_founder4_role_criticality</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G8" s="5">
         <f>B8*C8+D8+E8*100000+F8*50000</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H8" s="20">
         <f>IF($G$9=0,0,G8/$G$9*(1-in_esop_pool_pct))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -4684,7 +4684,7 @@
       </c>
       <c r="G9" s="5">
         <f>SUM(G5:G8)</f>
-        <v/>
+        <v>1200000</v>
       </c>
     </row>
     <row r="10">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="H10" s="20">
         <f>in_esop_pool_pct</f>
-        <v/>
+        <v>0.15</v>
       </c>
     </row>
     <row r="11">
@@ -4706,7 +4706,7 @@
       </c>
       <c r="H11" s="20">
         <f>SUM(H5:H8)+H10</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>